<commit_message>
feat: implementa ajustes e regras de negocio da ata de 21/08
- Move comparacao com outras tradings para o backlog
- Atualiza cadastro e calculo de pracas com matriz tributaria completa (Funrural, Imposto Base NF e Base UPF)
- Adiciona selecao de Campanha e Subcategoria no simulador
- Ajusta cashback de Barter como devolucao financeira (sem reducao fisica indevida na CPR)
- Adiciona calculo de sacas equivalentes nas modalidades financeiras (Syde, Fiso, Syngenta)
- Revisa formulas e tooltips de Custo Real Total e Custo Real da Operacao
- Adiciona ata pedidos de alteracoes 21 08.md
</commit_message>
<xml_diff>
--- a/Impostos 1.xlsx
+++ b/Impostos 1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://syngenta-my.sharepoint.com/personal/alessandra_monteiro_syngenta_com/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e0e760a1110f3163/Projetos/Barter Simulator/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2" documentId="8_{14D1CDE4-CD89-4227-8582-136824AFE95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D5AF57-F6F9-4F58-BA9D-BA833F426E02}"/>
@@ -298,9 +298,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
-    <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -355,7 +355,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -652,23 +652,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A78E500A-5AD6-458E-953B-06520C2567A9}">
   <dimension ref="A1:O25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7265625" customWidth="1"/>
+    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" style="5" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="4.140625" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.1796875" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="0" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7265625" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="34" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="48.28515625" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5703125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="48.26953125" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="13.54296875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -707,7 +707,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
@@ -743,7 +743,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>14</v>
       </c>
@@ -783,7 +783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
@@ -855,7 +855,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
@@ -891,7 +891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -927,7 +927,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>25</v>
       </c>
@@ -963,7 +963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>26</v>
       </c>
@@ -999,7 +999,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>29</v>
       </c>
@@ -1035,7 +1035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>30</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>31</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>32</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="K14" s="5" t="s">
         <v>29</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="K15" s="5" t="s">
         <v>30</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B16" s="10"/>
       <c r="C16" s="3"/>
       <c r="K16" s="5" t="s">
@@ -1200,7 +1200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="5"/>
       <c r="C17" s="13"/>
       <c r="K17" s="5" t="s">
@@ -1219,7 +1219,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="C18" s="13"/>
       <c r="K18" s="5" t="s">
         <v>31</v>
@@ -1237,7 +1237,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="K19" s="5" t="s">
         <v>32</v>
       </c>
@@ -1254,7 +1254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="29" x14ac:dyDescent="0.35">
       <c r="K20" s="14" t="s">
         <v>32</v>
       </c>
@@ -1271,13 +1271,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="K22" s="5"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="K23" s="5"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="K25" s="5"/>
     </row>
   </sheetData>

</xml_diff>